<commit_message>
testing different versions od code to extract data from pdf file
</commit_message>
<xml_diff>
--- a/data/tracker_files/file_status_record_2026-02-27.xlsx
+++ b/data/tracker_files/file_status_record_2026-02-27.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="656" uniqueCount="329">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="719" uniqueCount="336">
   <si>
     <t>Pipeline</t>
   </si>
@@ -1009,6 +1009,27 @@
   </si>
   <si>
     <t>Valley pipeline</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Files Available</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Tafiff selection</t>
+  </si>
+  <si>
+    <t>Last</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>Last -1</t>
   </si>
 </sst>
 </file>
@@ -1353,13 +1374,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:F131"/>
+  <dimension ref="A1:K131"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1378,8 +1399,14 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H1" t="s">
+        <v>330</v>
+      </c>
+      <c r="J1" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -1398,8 +1425,11 @@
       <c r="F2" s="1">
         <v>6.0296296296296291E-4</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H2" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -1418,8 +1448,11 @@
       <c r="F3" s="1">
         <v>5.3747685185185192E-4</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H3" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -1438,8 +1471,17 @@
       <c r="F4" s="1">
         <v>5.627199074074074E-4</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H4" t="s">
+        <v>331</v>
+      </c>
+      <c r="J4">
+        <v>4</v>
+      </c>
+      <c r="K4" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -1459,7 +1501,7 @@
         <v>5.2346064814814811E-4</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -1478,8 +1520,11 @@
       <c r="F6" s="1">
         <v>4.8365740740740742E-4</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H6" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>23</v>
       </c>
@@ -1498,8 +1543,11 @@
       <c r="F7" s="1">
         <v>5.3291666666666667E-4</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H7" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>26</v>
       </c>
@@ -1519,7 +1567,7 @@
         <v>5.1997685185185187E-4</v>
       </c>
     </row>
-    <row r="9" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>29</v>
       </c>
@@ -1539,7 +1587,7 @@
         <v>6.1215277777777776E-4</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>33</v>
       </c>
@@ -1558,8 +1606,17 @@
       <c r="F10" s="1">
         <v>5.224305555555555E-4</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H10" t="s">
+        <v>331</v>
+      </c>
+      <c r="J10">
+        <v>2</v>
+      </c>
+      <c r="K10" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>36</v>
       </c>
@@ -1578,8 +1635,11 @@
       <c r="F11" s="1">
         <v>5.2546296296296293E-4</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H11" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>39</v>
       </c>
@@ -1598,8 +1658,11 @@
       <c r="F12" s="1">
         <v>4.639814814814815E-4</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H12" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>42</v>
       </c>
@@ -1618,8 +1681,11 @@
       <c r="F13" s="1">
         <v>4.637037037037037E-4</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H13" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>45</v>
       </c>
@@ -1638,8 +1704,17 @@
       <c r="F14" s="1">
         <v>5.0509259259259257E-4</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H14" t="s">
+        <v>331</v>
+      </c>
+      <c r="J14">
+        <v>2</v>
+      </c>
+      <c r="K14" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>47</v>
       </c>
@@ -1658,8 +1733,14 @@
       <c r="F15" s="1">
         <v>5.1175925925925922E-4</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H15" t="s">
+        <v>331</v>
+      </c>
+      <c r="J15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>49</v>
       </c>
@@ -1678,8 +1759,14 @@
       <c r="F16" s="1">
         <v>5.1445601851851847E-4</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H16" t="s">
+        <v>331</v>
+      </c>
+      <c r="J16">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>52</v>
       </c>
@@ -1698,8 +1785,11 @@
       <c r="F17" s="1">
         <v>5.7585648148148144E-4</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H17" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>55</v>
       </c>
@@ -1718,8 +1808,14 @@
       <c r="F18" s="1">
         <v>5.1160879629629636E-4</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H18" t="s">
+        <v>331</v>
+      </c>
+      <c r="J18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>58</v>
       </c>
@@ -1738,8 +1834,14 @@
       <c r="F19" s="1">
         <v>5.3748842592592596E-4</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H19" t="s">
+        <v>331</v>
+      </c>
+      <c r="J19">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>60</v>
       </c>
@@ -1758,8 +1860,11 @@
       <c r="F20" s="1">
         <v>4.644675925925926E-4</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H20" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>63</v>
       </c>
@@ -1778,8 +1883,11 @@
       <c r="F21" s="1">
         <v>5.2137731481481479E-4</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H21" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>65</v>
       </c>
@@ -1798,8 +1906,14 @@
       <c r="F22" s="1">
         <v>5.1574074074074076E-4</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H22" t="s">
+        <v>331</v>
+      </c>
+      <c r="J22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>68</v>
       </c>
@@ -1818,8 +1932,14 @@
       <c r="F23" s="1">
         <v>6.0320601851851844E-4</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H23" t="s">
+        <v>331</v>
+      </c>
+      <c r="J23">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>71</v>
       </c>
@@ -1839,7 +1959,7 @@
         <v>5.2545138888888889E-4</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>74</v>
       </c>
@@ -1858,8 +1978,14 @@
       <c r="F25" s="1">
         <v>4.5834490740740742E-4</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H25" t="s">
+        <v>331</v>
+      </c>
+      <c r="J25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>77</v>
       </c>
@@ -1878,8 +2004,11 @@
       <c r="F26" s="1">
         <v>4.5928240740740738E-4</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H26" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>79</v>
       </c>
@@ -1898,8 +2027,14 @@
       <c r="F27" s="1">
         <v>4.8806712962962958E-4</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H27" t="s">
+        <v>331</v>
+      </c>
+      <c r="J27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>81</v>
       </c>
@@ -1919,7 +2054,7 @@
         <v>4.6723379629629632E-4</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>84</v>
       </c>
@@ -1938,8 +2073,17 @@
       <c r="F29" s="1">
         <v>4.7453703703703698E-4</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H29" t="s">
+        <v>331</v>
+      </c>
+      <c r="J29">
+        <v>2</v>
+      </c>
+      <c r="K29" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>87</v>
       </c>
@@ -1958,8 +2102,17 @@
       <c r="F30" s="1">
         <v>5.6005787037037038E-4</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H30" t="s">
+        <v>331</v>
+      </c>
+      <c r="J30">
+        <v>4</v>
+      </c>
+      <c r="K30" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>89</v>
       </c>
@@ -1978,8 +2131,17 @@
       <c r="F31" s="1">
         <v>5.2281249999999995E-4</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H31" t="s">
+        <v>331</v>
+      </c>
+      <c r="J31">
+        <v>2</v>
+      </c>
+      <c r="K31" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>92</v>
       </c>
@@ -1998,8 +2160,17 @@
       <c r="F32" s="1">
         <v>5.1497685185185186E-4</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H32" t="s">
+        <v>331</v>
+      </c>
+      <c r="J32">
+        <v>1</v>
+      </c>
+      <c r="K32" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>94</v>
       </c>
@@ -2018,8 +2189,17 @@
       <c r="F33" s="1">
         <v>5.4122685185185187E-4</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H33" t="s">
+        <v>331</v>
+      </c>
+      <c r="J33">
+        <v>3</v>
+      </c>
+      <c r="K33" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>97</v>
       </c>
@@ -2039,7 +2219,7 @@
         <v>5.1362268518518521E-4</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>99</v>
       </c>
@@ -2058,8 +2238,17 @@
       <c r="F35" s="1">
         <v>5.1724537037037038E-4</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H35" t="s">
+        <v>331</v>
+      </c>
+      <c r="J35">
+        <v>2</v>
+      </c>
+      <c r="K35" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>101</v>
       </c>
@@ -2078,8 +2267,17 @@
       <c r="F36" s="1">
         <v>5.259027777777778E-4</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H36" t="s">
+        <v>331</v>
+      </c>
+      <c r="J36">
+        <v>2</v>
+      </c>
+      <c r="K36" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>104</v>
       </c>
@@ -2099,7 +2297,7 @@
         <v>5.1111111111111105E-4</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>108</v>
       </c>
@@ -2118,8 +2316,11 @@
       <c r="F38" s="1">
         <v>4.6537037037037028E-4</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H38" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>110</v>
       </c>
@@ -2138,8 +2339,17 @@
       <c r="F39" s="1">
         <v>4.9482638888888894E-4</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H39" t="s">
+        <v>331</v>
+      </c>
+      <c r="J39">
+        <v>7</v>
+      </c>
+      <c r="K39" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>112</v>
       </c>
@@ -2158,8 +2368,11 @@
       <c r="F40" s="1">
         <v>5.1782407407407409E-4</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H40" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>115</v>
       </c>
@@ -2178,8 +2391,17 @@
       <c r="F41" s="1">
         <v>5.0766203703703704E-4</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H41" t="s">
+        <v>331</v>
+      </c>
+      <c r="J41">
+        <v>1</v>
+      </c>
+      <c r="K41" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>117</v>
       </c>
@@ -2198,8 +2420,14 @@
       <c r="F42" s="1">
         <v>5.1321759259259257E-4</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H42" t="s">
+        <v>331</v>
+      </c>
+      <c r="J42">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>119</v>
       </c>
@@ -2218,8 +2446,17 @@
       <c r="F43" s="1">
         <v>5.1107638888888882E-4</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H43" t="s">
+        <v>331</v>
+      </c>
+      <c r="J43">
+        <v>1</v>
+      </c>
+      <c r="K43" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>121</v>
       </c>
@@ -2238,8 +2475,17 @@
       <c r="F44" s="1">
         <v>5.209837962962963E-4</v>
       </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H44" t="s">
+        <v>331</v>
+      </c>
+      <c r="J44">
+        <v>1</v>
+      </c>
+      <c r="K44" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>123</v>
       </c>
@@ -2258,8 +2504,17 @@
       <c r="F45" s="1">
         <v>5.697685185185185E-4</v>
       </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H45" t="s">
+        <v>331</v>
+      </c>
+      <c r="J45">
+        <v>1</v>
+      </c>
+      <c r="K45" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>125</v>
       </c>
@@ -2278,8 +2533,11 @@
       <c r="F46" s="1">
         <v>5.5378472222222222E-4</v>
       </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H46" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>127</v>
       </c>
@@ -2298,8 +2556,17 @@
       <c r="F47" s="1">
         <v>5.3711805555555555E-4</v>
       </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H47" t="s">
+        <v>331</v>
+      </c>
+      <c r="J47">
+        <v>1</v>
+      </c>
+      <c r="K47" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>129</v>
       </c>
@@ -2318,8 +2585,17 @@
       <c r="F48" s="1">
         <v>5.176967592592593E-4</v>
       </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H48" t="s">
+        <v>331</v>
+      </c>
+      <c r="J48">
+        <v>1</v>
+      </c>
+      <c r="K48" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>131</v>
       </c>
@@ -2338,8 +2614,17 @@
       <c r="F49" s="1">
         <v>5.6923611111111118E-4</v>
       </c>
-    </row>
-    <row r="50" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H49" t="s">
+        <v>331</v>
+      </c>
+      <c r="J49">
+        <v>2</v>
+      </c>
+      <c r="K49" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>133</v>
       </c>
@@ -2359,7 +2644,7 @@
         <v>5.164351851851852E-4</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>136</v>
       </c>
@@ -2378,8 +2663,17 @@
       <c r="F51" s="1">
         <v>6.042708333333334E-4</v>
       </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H51" t="s">
+        <v>331</v>
+      </c>
+      <c r="J51">
+        <v>2</v>
+      </c>
+      <c r="K51" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>138</v>
       </c>
@@ -2399,7 +2693,7 @@
         <v>5.8293981481481478E-4</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>140</v>
       </c>
@@ -2419,7 +2713,7 @@
         <v>5.1318287037037033E-4</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>142</v>
       </c>
@@ -2439,7 +2733,7 @@
         <v>5.2935185185185181E-4</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>144</v>
       </c>
@@ -2459,7 +2753,7 @@
         <v>5.2660879629629629E-4</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>146</v>
       </c>
@@ -2479,7 +2773,7 @@
         <v>6.000925925925926E-4</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>148</v>
       </c>
@@ -2499,7 +2793,7 @@
         <v>5.2234953703703699E-4</v>
       </c>
     </row>
-    <row r="58" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>150</v>
       </c>
@@ -2519,7 +2813,7 @@
         <v>5.0745370370370376E-4</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>152</v>
       </c>
@@ -2539,7 +2833,7 @@
         <v>5.286111111111111E-4</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>154</v>
       </c>
@@ -2559,7 +2853,7 @@
         <v>5.1931712962962966E-4</v>
       </c>
     </row>
-    <row r="61" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>156</v>
       </c>
@@ -2579,7 +2873,7 @@
         <v>5.2248842592592592E-4</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>159</v>
       </c>
@@ -2599,7 +2893,7 @@
         <v>5.3643518518518515E-4</v>
       </c>
     </row>
-    <row r="63" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>162</v>
       </c>
@@ -2619,7 +2913,7 @@
         <v>5.2337962962962961E-4</v>
       </c>
     </row>
-    <row r="64" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>165</v>
       </c>

</xml_diff>